<commit_message>
feat: Add best practices for Supabase Postgres schema management
- Introduced guidelines for using lowercase identifiers to avoid case-sensitivity issues.
- Added recommendations for partitioning large tables to enhance performance.
- Provided strategies for selecting optimal primary key types to improve index locality and reduce fragmentation.
- Emphasized the principle of least privilege in security practices.
- Implemented row-level security (RLS) for multi-tenant data protection.
- Optimized RLS policies for better performance with strategic use of subqueries and indexes.
- Created a changelog for tracking changes and updates in the Supabase skill.
- Developed comprehensive documentation for the Supabase skill, including core principles and security checklists.
- Established a feedback mechanism for users to report issues with the skill's guidance.
- Added a skills lock file to manage dependencies and versions.
</commit_message>
<xml_diff>
--- a/exports/Master_B2B_Leads.xlsx
+++ b/exports/Master_B2B_Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="195">
   <si>
     <t>Company Name</t>
   </si>
@@ -61,43 +61,358 @@
     <t>Scraped Date</t>
   </si>
   <si>
-    <t>- P A L M E R A -</t>
-  </si>
-  <si>
-    <t>916627939</t>
+    <t>The Steward Shipping Foundation</t>
+  </si>
+  <si>
+    <t>19871120103</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>1951-05-08</t>
+  </si>
+  <si>
+    <t>DNC</t>
+  </si>
+  <si>
+    <t>133 County Rd 17, Suite E2A, Elizabeth, CO, 80107, USA</t>
+  </si>
+  <si>
+    <t>Elizabeth</t>
+  </si>
+  <si>
+    <t>80107</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Jurisdiction: CO</t>
+  </si>
+  <si>
+    <t>US Socrata Open Data (Colorado &amp; NY)</t>
+  </si>
+  <si>
+    <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>THE STANDARD SHALE PRODUCTS COMPANY</t>
+  </si>
+  <si>
+    <t>19871069482</t>
+  </si>
+  <si>
+    <t>1919-05-26</t>
+  </si>
+  <si>
+    <t>DPC</t>
+  </si>
+  <si>
+    <t>925 N Eldridge Pkwy, Houston, TX, 77079, USA</t>
+  </si>
+  <si>
+    <t>Houston</t>
+  </si>
+  <si>
+    <t>77079</t>
+  </si>
+  <si>
+    <t>INEXCO OIL COMPANY</t>
+  </si>
+  <si>
+    <t>19871045781</t>
+  </si>
+  <si>
+    <t>1968-06-24</t>
+  </si>
+  <si>
+    <t>FPC</t>
+  </si>
+  <si>
+    <t>Jurisdiction: DE</t>
+  </si>
+  <si>
+    <t>CONOCOPHILLIPS COMMUNICAITONS INC.</t>
+  </si>
+  <si>
+    <t>19871041580</t>
+  </si>
+  <si>
+    <t>1964-07-29</t>
+  </si>
+  <si>
+    <t>CONTINENTAL OIL COMPANY</t>
+  </si>
+  <si>
+    <t>19871039367</t>
+  </si>
+  <si>
+    <t>1967-04-03</t>
+  </si>
+  <si>
+    <t>AMERICAN ASIATIC SHIPPING AGEN CIES SDN. BHD.</t>
+  </si>
+  <si>
+    <t>194600008E</t>
+  </si>
+  <si>
+    <t>Singapore</t>
+  </si>
+  <si>
+    <t>Dissolved - Members Voluntary Winding Up</t>
+  </si>
+  <si>
+    <t>1946-08-14</t>
+  </si>
+  <si>
+    <t>Exempt Private Company Limited by Shares</t>
+  </si>
+  <si>
+    <t>Blk 75 TANGLIN ROAD, Singapore 247917</t>
+  </si>
+  <si>
+    <t>247917</t>
+  </si>
+  <si>
+    <t>6 Officers Registered</t>
+  </si>
+  <si>
+    <t>52222</t>
+  </si>
+  <si>
+    <t>ACRA (data.gov.sg)</t>
+  </si>
+  <si>
+    <t>ANEKA SERVICES</t>
+  </si>
+  <si>
+    <t>10789100W</t>
+  </si>
+  <si>
+    <t>Live</t>
+  </si>
+  <si>
+    <t>1975-07-29</t>
+  </si>
+  <si>
+    <t>Sole Proprietorship/ Partnership</t>
+  </si>
+  <si>
+    <t>Blk 19 JALAN TENTERAM, Singapore 321019</t>
+  </si>
+  <si>
+    <t>321019</t>
+  </si>
+  <si>
+    <t>3 Officers Registered</t>
+  </si>
+  <si>
+    <t>78104</t>
+  </si>
+  <si>
+    <t>ALKEMAL SHIPPING ORGANISATION</t>
+  </si>
+  <si>
+    <t>07608100A</t>
+  </si>
+  <si>
+    <t>Terminated</t>
+  </si>
+  <si>
+    <t>1975-05-13</t>
+  </si>
+  <si>
+    <t>Blk 90 CECIL STREET RHB BANK BUILDING, Singapore 069531</t>
+  </si>
+  <si>
+    <t>069531</t>
+  </si>
+  <si>
+    <t>2 Officers Registered</t>
+  </si>
+  <si>
+    <t>52224</t>
+  </si>
+  <si>
+    <t>ADI SHIPPING</t>
+  </si>
+  <si>
+    <t>07364700D</t>
+  </si>
+  <si>
+    <t>1975-04-11</t>
+  </si>
+  <si>
+    <t>Blk 342 ONAN ROAD, Singapore 424734</t>
+  </si>
+  <si>
+    <t>424734</t>
+  </si>
+  <si>
+    <t>ABADI SHIPPING COMPANY</t>
+  </si>
+  <si>
+    <t>05628000M</t>
+  </si>
+  <si>
+    <t>1975-02-04</t>
+  </si>
+  <si>
+    <t>Blk 48 BOAT QUAY, Singapore 049837</t>
+  </si>
+  <si>
+    <t>049837</t>
+  </si>
+  <si>
+    <t>SOGESTRAN SHIPPING</t>
+  </si>
+  <si>
+    <t>831375092</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>2017-08-01</t>
+  </si>
+  <si>
+    <t>5710</t>
+  </si>
+  <si>
+    <t>11 RUE, 76600, LE HAVRE, France</t>
+  </si>
+  <si>
+    <t>LE HAVRE</t>
+  </si>
+  <si>
+    <t>76600</t>
+  </si>
+  <si>
+    <t>BENOIST FRANCOIS PIERRE MARIE GROSJEAN (Directeur Général)</t>
+  </si>
+  <si>
+    <t>64.20Z</t>
+  </si>
+  <si>
+    <t>Recherche d'entreprises (api.gouv.fr)</t>
+  </si>
+  <si>
+    <t>SEA INVEST SHIPPING AGENCY (FRANCOIS BOYER DE LA GIRODAY - MUSO)</t>
+  </si>
+  <si>
+    <t>319116661</t>
+  </si>
+  <si>
+    <t>1980-09-01</t>
+  </si>
+  <si>
+    <t>BOULEVARD, 76530, GRAND-COURONNE, France</t>
+  </si>
+  <si>
+    <t>GRAND-COURONNE</t>
+  </si>
+  <si>
+    <t>76530</t>
+  </si>
+  <si>
+    <t>FLORENT ARCHANGE CLAUDE MASSART (Président de SAS)</t>
+  </si>
+  <si>
+    <t>52.22Z</t>
+  </si>
+  <si>
+    <t>BALIER SHIPPING</t>
+  </si>
+  <si>
+    <t>904629078</t>
+  </si>
+  <si>
+    <t>2021-11-01</t>
+  </si>
+  <si>
+    <t>25 ROUTE, 64220, AINCILLE, France</t>
+  </si>
+  <si>
+    <t>AINCILLE</t>
+  </si>
+  <si>
+    <t>64220</t>
+  </si>
+  <si>
+    <t>CHARLES MARCEL JEAN BALIER (Président de SAS)</t>
+  </si>
+  <si>
+    <t>BBL SHIPPING</t>
+  </si>
+  <si>
+    <t>056802572</t>
+  </si>
+  <si>
+    <t>1956-01-01</t>
+  </si>
+  <si>
+    <t>31 RUE, 77600, BUSSY-SAINT-GEORGES, France</t>
+  </si>
+  <si>
+    <t>BUSSY-SAINT-GEORGES</t>
+  </si>
+  <si>
+    <t>77600</t>
+  </si>
+  <si>
+    <t>MARC LINDER (Commissaire aux comptes suppléant)</t>
+  </si>
+  <si>
+    <t>52.29B</t>
+  </si>
+  <si>
+    <t>T ET T SHIPPING</t>
+  </si>
+  <si>
+    <t>478908262</t>
+  </si>
+  <si>
+    <t>2004-09-23</t>
+  </si>
+  <si>
+    <t>CHEMIN, 13200, ARLES, France</t>
+  </si>
+  <si>
+    <t>ARLES</t>
+  </si>
+  <si>
+    <t>13200</t>
+  </si>
+  <si>
+    <t>TETYANA GALIBERT (BALATS'KA) (Président de SAS)</t>
+  </si>
+  <si>
+    <t>KODAL SHIPPING</t>
+  </si>
+  <si>
+    <t>914019281</t>
   </si>
   <si>
     <t>Norway</t>
   </si>
   <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>2016-01-26</t>
+    <t>2014-08-19</t>
   </si>
   <si>
     <t>Forening/lag/innretning</t>
   </si>
   <si>
-    <t>Strandgaten 208, 5004, BERGEN, Norge</t>
-  </si>
-  <si>
-    <t>BERGEN</t>
-  </si>
-  <si>
-    <t>5004</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>https://palmera-i-bergen.no</t>
-  </si>
-  <si>
-    <t>palmera.i.bergen@gmail.com</t>
-  </si>
-  <si>
-    <t>451 72 987</t>
+    <t>Solløkkasvingen 16, 3233, SANDEFJORD, Norge</t>
+  </si>
+  <si>
+    <t>SANDEFJORD</t>
+  </si>
+  <si>
+    <t>3233</t>
   </si>
   <si>
     <t>Aktiviteter i andre medlemsorganisasjoner ellers</t>
@@ -106,346 +421,181 @@
     <t>Brønnøysundregistrene (data.brreg.no)</t>
   </si>
   <si>
-    <t>2026-10-11</t>
-  </si>
-  <si>
-    <t>- ZOTKO .NO</t>
-  </si>
-  <si>
-    <t>933365573</t>
-  </si>
-  <si>
-    <t>2024-04-25</t>
+    <t>HBV SHIPPING</t>
+  </si>
+  <si>
+    <t>913155262</t>
+  </si>
+  <si>
+    <t>2014-02-27</t>
+  </si>
+  <si>
+    <t>Vannøyaveien 31, 3231, SANDEFJORD, Norge</t>
+  </si>
+  <si>
+    <t>3231</t>
+  </si>
+  <si>
+    <t>https://hbvshipping.com</t>
+  </si>
+  <si>
+    <t>post@hbvshipping.com</t>
+  </si>
+  <si>
+    <t>995 09 394</t>
+  </si>
+  <si>
+    <t>FJELLSTAD SHIPPING</t>
+  </si>
+  <si>
+    <t>914331242</t>
+  </si>
+  <si>
+    <t>2015-03-26</t>
   </si>
   <si>
     <t>Enkeltpersonforetak</t>
   </si>
   <si>
-    <t>Follerøvegen 20, 6652, SURNADAL, Norge</t>
-  </si>
-  <si>
-    <t>SURNADAL</t>
-  </si>
-  <si>
-    <t>6652</t>
-  </si>
-  <si>
-    <t>Detaljhandel med drikkevarer</t>
-  </si>
-  <si>
-    <t>----ADVOKATFIRMAET CATO MYHRE</t>
-  </si>
-  <si>
-    <t>934551435</t>
-  </si>
-  <si>
-    <t>2024-11-27</t>
-  </si>
-  <si>
-    <t>Grimelundshaugen 33, 0374, OSLO, Norge</t>
+    <t>c/o Beatrix Goovaerts Fjellstad, Vibes gate 24, 0356, OSLO, Norge</t>
   </si>
   <si>
     <t>OSLO</t>
   </si>
   <si>
-    <t>0374</t>
-  </si>
-  <si>
-    <t>92096030</t>
-  </si>
-  <si>
-    <t>Juridisk tjenesteyting</t>
-  </si>
-  <si>
-    <t>-EBE- DATA Eyolf Berg</t>
-  </si>
-  <si>
-    <t>988539473</t>
-  </si>
-  <si>
-    <t>2005-08-20</t>
-  </si>
-  <si>
-    <t>Bekkeliveien 5, 3470, SLEMMESTAD, Norge</t>
-  </si>
-  <si>
-    <t>SLEMMESTAD</t>
-  </si>
-  <si>
-    <t>3470</t>
-  </si>
-  <si>
-    <t>https://www.ebe-data.com</t>
-  </si>
-  <si>
-    <t>ebe@ebe-data.com</t>
-  </si>
-  <si>
-    <t>911 76 537</t>
-  </si>
-  <si>
-    <t>Konsulentvirksomhet tilknyttet informasjonsteknologi og forvaltning og drift av it-systemer</t>
-  </si>
-  <si>
-    <t>-G- GROUP AS</t>
-  </si>
-  <si>
-    <t>989061593</t>
-  </si>
-  <si>
-    <t>2006-01-23</t>
-  </si>
-  <si>
-    <t>Aksjeselskap</t>
-  </si>
-  <si>
-    <t>c/o Gjørva, Hellerud gårdsvei 5B, 0671, OSLO, Norge</t>
-  </si>
-  <si>
-    <t>0671</t>
-  </si>
-  <si>
-    <t>TECH</t>
-  </si>
-  <si>
-    <t>525245759</t>
-  </si>
-  <si>
-    <t>France</t>
-  </si>
-  <si>
-    <t>2010-10-01</t>
-  </si>
-  <si>
-    <t>5710</t>
-  </si>
-  <si>
-    <t>34 AVENUE, 75008, PARIS, France</t>
+    <t>0356</t>
+  </si>
+  <si>
+    <t>felix.gf@me.com</t>
+  </si>
+  <si>
+    <t>94169203</t>
+  </si>
+  <si>
+    <t>Annen forretningsmessig tjenesteyting ikke nevnt annet sted</t>
+  </si>
+  <si>
+    <t>AUBY SHIPPING</t>
+  </si>
+  <si>
+    <t>937336292</t>
+  </si>
+  <si>
+    <t>2026-03-18</t>
+  </si>
+  <si>
+    <t>Silkestråveien 17, 3261, LARVIK, Norge</t>
+  </si>
+  <si>
+    <t>LARVIK</t>
+  </si>
+  <si>
+    <t>3261</t>
+  </si>
+  <si>
+    <t>Fiske og fangst i sjø</t>
+  </si>
+  <si>
+    <t>ARTHUR SHIPPING</t>
+  </si>
+  <si>
+    <t>929585909</t>
+  </si>
+  <si>
+    <t>2022-08-02</t>
+  </si>
+  <si>
+    <t>Søster Mathildes gate 20A, 1461, LØRENSKOG, Norge</t>
+  </si>
+  <si>
+    <t>LØRENSKOG</t>
+  </si>
+  <si>
+    <t>1461</t>
+  </si>
+  <si>
+    <t>Formidlingstjenester tilknyttet godstransport via skip</t>
+  </si>
+  <si>
+    <t>Summit Surgical Technologies LLC</t>
+  </si>
+  <si>
+    <t>20081620713</t>
+  </si>
+  <si>
+    <t>2008-11-29</t>
+  </si>
+  <si>
+    <t>DLLC</t>
+  </si>
+  <si>
+    <t>2525 S Dayton Way Apt 1210, Denver, CO, 80231, USA</t>
+  </si>
+  <si>
+    <t>Denver</t>
+  </si>
+  <si>
+    <t>80231</t>
+  </si>
+  <si>
+    <t>ASIA ELECTRONIC ENGINEERING TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>06912200L</t>
+  </si>
+  <si>
+    <t>Blk 443 ANG MO KIO AVENUE 10, Singapore 560443</t>
+  </si>
+  <si>
+    <t>560443</t>
+  </si>
+  <si>
+    <t>95299</t>
+  </si>
+  <si>
+    <t>TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>440708717</t>
+  </si>
+  <si>
+    <t>2002-02-01</t>
+  </si>
+  <si>
+    <t>5499</t>
+  </si>
+  <si>
+    <t>80 RUE, 75017, PARIS, France</t>
   </si>
   <si>
     <t>PARIS</t>
   </si>
   <si>
-    <t>75008</t>
-  </si>
-  <si>
-    <t>KLARA (Président de SAS)</t>
-  </si>
-  <si>
-    <t>35.11Z</t>
-  </si>
-  <si>
-    <t>Recherche d'entreprises (api.gouv.fr)</t>
-  </si>
-  <si>
-    <t>920686920</t>
-  </si>
-  <si>
-    <t>2022-10-20</t>
-  </si>
-  <si>
-    <t>6540</t>
-  </si>
-  <si>
-    <t>27 RUE, 17120, GREZAC, France</t>
-  </si>
-  <si>
-    <t>GREZAC</t>
-  </si>
-  <si>
-    <t>17120</t>
-  </si>
-  <si>
-    <t>EMILIE VIVIEN (CHARBONNEAU) (Gérant et associé indéfiniment responsable)</t>
-  </si>
-  <si>
-    <t>68.20B</t>
-  </si>
-  <si>
-    <t>908337132</t>
-  </si>
-  <si>
-    <t>2021-01-04</t>
-  </si>
-  <si>
-    <t>5202</t>
-  </si>
-  <si>
-    <t>32, 97190, LE GOSIER, France</t>
-  </si>
-  <si>
-    <t>LE GOSIER</t>
-  </si>
-  <si>
-    <t>97190</t>
-  </si>
-  <si>
-    <t>DIANA CAROLE SUZE-JOHNS (SUZE) (Autre)</t>
-  </si>
-  <si>
-    <t>443780580</t>
-  </si>
-  <si>
-    <t>2002-09-25</t>
-  </si>
-  <si>
-    <t>5499</t>
-  </si>
-  <si>
-    <t>500 ALLEE, 26300, BOURG-DE-PEAGE, France</t>
-  </si>
-  <si>
-    <t>BOURG-DE-PEAGE</t>
-  </si>
-  <si>
-    <t>26300</t>
-  </si>
-  <si>
-    <t>DANIEL VULIN (Gérant)</t>
-  </si>
-  <si>
-    <t>71.20B</t>
-  </si>
-  <si>
-    <t>479350464</t>
-  </si>
-  <si>
-    <t>2004-10-18</t>
-  </si>
-  <si>
-    <t>151 CHEMIN, 01320, VILLETTE-SUR-AIN, France</t>
-  </si>
-  <si>
-    <t>VILLETTE-SUR-AIN</t>
-  </si>
-  <si>
-    <t>01320</t>
-  </si>
-  <si>
-    <t>CHRISTOPHE CLAUDE CHABERT (Gérant)</t>
-  </si>
-  <si>
-    <t>70.10Z</t>
-  </si>
-  <si>
-    <t>AIK CHE HIONG</t>
-  </si>
-  <si>
-    <t>00733000J</t>
-  </si>
-  <si>
-    <t>Singapore</t>
-  </si>
-  <si>
-    <t>Live</t>
-  </si>
-  <si>
-    <t>1974-11-02</t>
-  </si>
-  <si>
-    <t>Sole Proprietorship/ Partnership</t>
-  </si>
-  <si>
-    <t>Blk 1 ANG MO KIO INDUSTRIAL PARK 2A AMK TECH I, Singapore 568049</t>
-  </si>
-  <si>
-    <t>568049</t>
-  </si>
-  <si>
-    <t>3 Officers Registered</t>
-  </si>
-  <si>
-    <t>MANUFACTURED JOSS STICK</t>
-  </si>
-  <si>
-    <t>ACRA (data.gov.sg)</t>
-  </si>
-  <si>
-    <t>ASIA HEALTH EQUIPMENT (PRIVATE) LIMITED</t>
-  </si>
-  <si>
-    <t>197100458E</t>
-  </si>
-  <si>
-    <t>Struck Off</t>
-  </si>
-  <si>
-    <t>1971-05-04</t>
-  </si>
-  <si>
-    <t>Exempt Private Company Limited by Shares</t>
-  </si>
-  <si>
-    <t>12 Officers Registered</t>
-  </si>
-  <si>
-    <t>46441</t>
-  </si>
-  <si>
-    <t>ADVISORY &amp; TECHNICAL MARINE SERVICES PTE LTD</t>
-  </si>
-  <si>
-    <t>197400150E</t>
-  </si>
-  <si>
-    <t>1974-01-31</t>
-  </si>
-  <si>
-    <t>Blk 896 DUNEARN ROAD LINK@896, Singapore 589472</t>
-  </si>
-  <si>
-    <t>589472</t>
-  </si>
-  <si>
-    <t>14 Officers Registered</t>
-  </si>
-  <si>
-    <t>MARINE TECH CONSULTANTS/SURVERYORS, ARRANGE SHIP REPAIRS, SUPPLY SHIP SPARES</t>
-  </si>
-  <si>
-    <t>A.B.C. ENGINEERING PTE. LTD.</t>
-  </si>
-  <si>
-    <t>197600154R</t>
-  </si>
-  <si>
-    <t>Live Company</t>
-  </si>
-  <si>
-    <t>1976-01-22</t>
-  </si>
-  <si>
-    <t>Blk 5 ANG MO KIO INDUSTRIAL PARK 2A AMK TECH II, Singapore 567760</t>
-  </si>
-  <si>
-    <t>567760</t>
-  </si>
-  <si>
-    <t>15 Officers Registered</t>
-  </si>
-  <si>
-    <t>30110</t>
-  </si>
-  <si>
-    <t>AIR-TECH INDUSTRIES PTE LTD</t>
-  </si>
-  <si>
-    <t>197900484H</t>
-  </si>
-  <si>
-    <t>Dissolved - Compulsory Winding Up (Insolvency)</t>
-  </si>
-  <si>
-    <t>1979-02-22</t>
-  </si>
-  <si>
-    <t>Blk 158 GUL CIRCLE, Singapore 629615</t>
-  </si>
-  <si>
-    <t>629615</t>
-  </si>
-  <si>
-    <t>MANUF/REPAIR NON-ELECT MACHINERY/EQUIPMENT NEC</t>
+    <t>75017</t>
+  </si>
+  <si>
+    <t>51.4F</t>
+  </si>
+  <si>
+    <t>AVALOS TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>919544635</t>
+  </si>
+  <si>
+    <t>2017-09-11</t>
+  </si>
+  <si>
+    <t>Sjåberg 14, 5516, HAUGESUND, Norge</t>
+  </si>
+  <si>
+    <t>HAUGESUND</t>
+  </si>
+  <si>
+    <t>5516</t>
+  </si>
+  <si>
+    <t>Dataprogrammeringstjenester</t>
   </si>
 </sst>
 </file>
@@ -876,21 +1026,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="45" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
     <col min="7" max="7" width="45" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="8" max="8" width="23" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
     <col min="10" max="10" width="45" customWidth="1"/>
-    <col min="11" max="11" width="31" customWidth="1"/>
-    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="11" max="11" width="27" customWidth="1"/>
+    <col min="12" max="12" width="24" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
     <col min="14" max="14" width="45" customWidth="1"/>
     <col min="15" max="15" width="41" customWidth="1"/>
@@ -979,30 +1129,30 @@
         <v>25</v>
       </c>
       <c r="K2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>18</v>
@@ -1011,20 +1161,20 @@
         <v>19</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>38</v>
-      </c>
       <c r="J3" s="3" t="s">
         <v>25</v>
       </c>
@@ -1038,21 +1188,21 @@
         <v>25</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
@@ -1061,20 +1211,20 @@
         <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="J4" s="2" t="s">
         <v>25</v>
       </c>
@@ -1085,24 +1235,24 @@
         <v>25</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>18</v>
@@ -1111,48 +1261,48 @@
         <v>19</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="F5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>53</v>
-      </c>
       <c r="J5" s="3" t="s">
         <v>25</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>18</v>
@@ -1161,19 +1311,19 @@
         <v>19</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>25</v>
@@ -1188,45 +1338,45 @@
         <v>25</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>25</v>
@@ -1238,95 +1388,95 @@
         <v>25</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="J8" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="O8" s="2" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>25</v>
@@ -1338,45 +1488,45 @@
         <v>25</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>25</v>
@@ -1388,45 +1538,45 @@
         <v>25</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>101</v>
+        <v>49</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>25</v>
@@ -1438,45 +1588,45 @@
         <v>25</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>108</v>
+        <v>19</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>25</v>
@@ -1488,45 +1638,45 @@
         <v>25</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>118</v>
+        <v>19</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>25</v>
@@ -1538,45 +1688,45 @@
         <v>25</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>126</v>
-      </c>
       <c r="H14" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>25</v>
@@ -1588,45 +1738,45 @@
         <v>25</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>129</v>
+        <v>103</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>132</v>
+        <v>19</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>25</v>
@@ -1638,63 +1788,513 @@
         <v>25</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="P17" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="F18" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="J18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K18" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G16" s="2" t="s">
+      <c r="L18" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="I16" s="2" t="s">
+      <c r="M18" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="N18" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="O16" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="P16" s="2" t="s">
-        <v>31</v>
+      <c r="D19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="M19" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="N19" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="O19" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="P19" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="N21" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="O21" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="P21" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="O22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="M23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="N23" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="O23" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="P23" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="O24" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="P24" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="N25" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="O25" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="P25" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update Master_B2B_Leads.xlsx with new data
</commit_message>
<xml_diff>
--- a/exports/Master_B2B_Leads.xlsx
+++ b/exports/Master_B2B_Leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="441">
   <si>
     <t>Company Name</t>
   </si>
@@ -61,18 +61,825 @@
     <t>Scraped Date</t>
   </si>
   <si>
+    <t>Global Connect Technologies LLC</t>
+  </si>
+  <si>
+    <t>20268168232</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>2026-09-22</t>
+  </si>
+  <si>
+    <t>DLLC</t>
+  </si>
+  <si>
+    <t>3100 Pearl PKWY, Boulder, CO, 80301, USA</t>
+  </si>
+  <si>
+    <t>Boulder</t>
+  </si>
+  <si>
+    <t>80301</t>
+  </si>
+  <si>
+    <t>Sina Ahandoust (Registered Agent)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Jurisdiction: CO</t>
+  </si>
+  <si>
+    <t>US Socrata Open Data (Colorado &amp; NY)</t>
+  </si>
+  <si>
+    <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>Generative Technology Corporation</t>
+  </si>
+  <si>
+    <t>20261073156</t>
+  </si>
+  <si>
+    <t>2026-01-22</t>
+  </si>
+  <si>
+    <t>FPC</t>
+  </si>
+  <si>
+    <t>540 Madison Ave Ste 20B, New York, NY, 10022, USA</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>10022</t>
+  </si>
+  <si>
+    <t>Jurisdiction: DE</t>
+  </si>
+  <si>
+    <t>ORBIT TECHNOLOGY LLC</t>
+  </si>
+  <si>
+    <t>20258160963</t>
+  </si>
+  <si>
+    <t>2025-10-24</t>
+  </si>
+  <si>
+    <t>17200 E Iliff Ave Ste A12 #135, Aurora, CO, 80013, USA</t>
+  </si>
+  <si>
+    <t>Aurora</t>
+  </si>
+  <si>
+    <t>80013</t>
+  </si>
+  <si>
+    <t>OPENQUANTUM TECHNOLOGY LLC</t>
+  </si>
+  <si>
+    <t>20258132420</t>
+  </si>
+  <si>
+    <t>2025-10-16</t>
+  </si>
+  <si>
+    <t>2525 Arapahoe Ave Ste E4 #1135, Boulder, CO, 80302, USA</t>
+  </si>
+  <si>
+    <t>80302</t>
+  </si>
+  <si>
+    <t>Ark Land LLC</t>
+  </si>
+  <si>
+    <t>19871046661</t>
+  </si>
+  <si>
+    <t>1970-09-04</t>
+  </si>
+  <si>
+    <t>FLLC</t>
+  </si>
+  <si>
+    <t>275 Technology Dr Ste 101, Canonsburg, PA, 15317, USA</t>
+  </si>
+  <si>
+    <t>Canonsburg</t>
+  </si>
+  <si>
+    <t>15317</t>
+  </si>
+  <si>
+    <t>Overwatch Technologies LLC</t>
+  </si>
+  <si>
+    <t>20228070748</t>
+  </si>
+  <si>
+    <t>2022-10-30</t>
+  </si>
+  <si>
+    <t>6760 Corporate Dr Ste 100, Colorado Springs, CO, 80919, USA</t>
+  </si>
+  <si>
+    <t>Colorado Springs</t>
+  </si>
+  <si>
+    <t>80919</t>
+  </si>
+  <si>
+    <t>DOUGLAS LYNN ECKELS (Registered Agent)</t>
+  </si>
+  <si>
+    <t>CLR Analytics Inc.</t>
+  </si>
+  <si>
+    <t>20201873629</t>
+  </si>
+  <si>
+    <t>2020-10-07</t>
+  </si>
+  <si>
+    <t>216 Technology Drive, Suite G, Irvine, CA, 92618, USA</t>
+  </si>
+  <si>
+    <t>Irvine</t>
+  </si>
+  <si>
+    <t>92618</t>
+  </si>
+  <si>
+    <t>Jurisdiction: United States</t>
+  </si>
+  <si>
+    <t>Big Dot of Happiness, LLC</t>
+  </si>
+  <si>
+    <t>20201015370</t>
+  </si>
+  <si>
+    <t>2020-01-06</t>
+  </si>
+  <si>
+    <t>412 Technology Dr, Menomonie, WI, 54751, USA</t>
+  </si>
+  <si>
+    <t>Menomonie</t>
+  </si>
+  <si>
+    <t>54751</t>
+  </si>
+  <si>
+    <t>Jurisdiction: WI</t>
+  </si>
+  <si>
+    <t>Transworld Technologies Inc.</t>
+  </si>
+  <si>
+    <t>20131594646</t>
+  </si>
+  <si>
+    <t>2013-10-16</t>
+  </si>
+  <si>
+    <t>1899 Wynkoop St Ste 275, Denver, CO, 80202, USA</t>
+  </si>
+  <si>
+    <t>Denver</t>
+  </si>
+  <si>
+    <t>80202</t>
+  </si>
+  <si>
+    <t>ASIASOURCE TECHNOLOGY PTE LTD</t>
+  </si>
+  <si>
+    <t>198004856H</t>
+  </si>
+  <si>
+    <t>Singapore</t>
+  </si>
+  <si>
+    <t>Struck Off</t>
+  </si>
+  <si>
+    <t>1980-12-27</t>
+  </si>
+  <si>
+    <t>Private Company Limited by Shares</t>
+  </si>
+  <si>
+    <t>Blk 203 HENDERSON ROAD HENDERSON INDUSTRIAL PARK, Singapore 159546</t>
+  </si>
+  <si>
+    <t>159546</t>
+  </si>
+  <si>
+    <t>16 Officers Registered</t>
+  </si>
+  <si>
+    <t>TRADING OF GEMOLOGICAL INSTRUMENTS</t>
+  </si>
+  <si>
+    <t>ACRA (data.gov.sg)</t>
+  </si>
+  <si>
+    <t>AIRESEARCH TECHNOLOGY PTE LTD</t>
+  </si>
+  <si>
+    <t>198003159D</t>
+  </si>
+  <si>
+    <t>Live Company</t>
+  </si>
+  <si>
+    <t>1980-09-04</t>
+  </si>
+  <si>
+    <t>Exempt Private Company Limited by Shares</t>
+  </si>
+  <si>
+    <t>Blk 9 TAGORE LANE 9 @ TAGORE, Singapore 787472</t>
+  </si>
+  <si>
+    <t>787472</t>
+  </si>
+  <si>
+    <t>17 Officers Registered</t>
+  </si>
+  <si>
+    <t>MFG &amp; REPAIR OF AIR PURIFICATION AND STERILISATION, AIR-CON &amp; VENTILATING EQPT</t>
+  </si>
+  <si>
+    <t>APPLIED SATELLITE TECHNOLOGY ASIA PTE. LTD.</t>
+  </si>
+  <si>
+    <t>198002772D</t>
+  </si>
+  <si>
+    <t>1980-08-04</t>
+  </si>
+  <si>
+    <t>Blk 110 LORONG 23 GEYLANG VICTORY CENTRE, Singapore 388410</t>
+  </si>
+  <si>
+    <t>388410</t>
+  </si>
+  <si>
+    <t>21 Officers Registered</t>
+  </si>
+  <si>
+    <t>DEAL &amp; DISTRIBUTE IMMARTSATE SATELLITE COMM &amp; SYS &amp; SVS FOR MARINE &amp; LAND USE</t>
+  </si>
+  <si>
+    <t>A.I. TECHNOLOGY PTE LTD</t>
+  </si>
+  <si>
+    <t>198001106N</t>
+  </si>
+  <si>
+    <t>1980-04-03</t>
+  </si>
+  <si>
+    <t>Blk 2 GUOK AVENUE, Singapore 119632</t>
+  </si>
+  <si>
+    <t>119632</t>
+  </si>
+  <si>
+    <t>14 Officers Registered</t>
+  </si>
+  <si>
+    <t>62021</t>
+  </si>
+  <si>
+    <t>ASIACLOUD SOLUTIONS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>197800982R</t>
+  </si>
+  <si>
+    <t>1978-05-02</t>
+  </si>
+  <si>
+    <t>Blk 18 HOWARD ROAD NOVELTY BIZCENTRE, Singapore 369585</t>
+  </si>
+  <si>
+    <t>369585</t>
+  </si>
+  <si>
+    <t>23 Officers Registered</t>
+  </si>
+  <si>
+    <t>IT CORP. RESELLER,SERVICING,NETWORK MAINT.,SOFTWARE DEV.,SYSTEM INTEGRATOR</t>
+  </si>
+  <si>
+    <t>ADVANCED CONCEPT TECHNOLOGY PTE. LTD.</t>
+  </si>
+  <si>
+    <t>197702591H</t>
+  </si>
+  <si>
+    <t>Dissolved - Compulsory Winding Up (Insolvency)</t>
+  </si>
+  <si>
+    <t>1977-11-28</t>
+  </si>
+  <si>
+    <t>Blk 1 TECK LIM ROAD, Singapore 088379</t>
+  </si>
+  <si>
+    <t>088379</t>
+  </si>
+  <si>
+    <t>9 Officers Registered</t>
+  </si>
+  <si>
+    <t>71129</t>
+  </si>
+  <si>
+    <t>ALLIANCE TECHNOLOGY AND DEVELOPMENT LIMITED</t>
+  </si>
+  <si>
+    <t>197200994H</t>
+  </si>
+  <si>
+    <t>1972-07-28</t>
+  </si>
+  <si>
+    <t>Public Company Limited by Shares</t>
+  </si>
+  <si>
+    <t>Blk 1 RAFFLES QUAY, Singapore 048583</t>
+  </si>
+  <si>
+    <t>048583</t>
+  </si>
+  <si>
+    <t>48 Officers Registered</t>
+  </si>
+  <si>
+    <t>HOLDING COMPANIES</t>
+  </si>
+  <si>
+    <t>ACE PLASTIC TECHNOLOGY PTE LTD</t>
+  </si>
+  <si>
+    <t>195800012E</t>
+  </si>
+  <si>
+    <t>1958-01-15</t>
+  </si>
+  <si>
+    <t>Blk 159 GUL CIRCLE, Singapore 629617</t>
+  </si>
+  <si>
+    <t>629617</t>
+  </si>
+  <si>
+    <t>64202</t>
+  </si>
+  <si>
+    <t>ARNOLD MEYER</t>
+  </si>
+  <si>
+    <t>09369300A</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
+  </si>
+  <si>
+    <t>1975-09-16</t>
+  </si>
+  <si>
+    <t>Sole Proprietorship/ Partnership</t>
+  </si>
+  <si>
+    <t>Blk 3 DUNSFOLD DRIVE DUNSFOLD RESIDENCES, Singapore 359366</t>
+  </si>
+  <si>
+    <t>359366</t>
+  </si>
+  <si>
+    <t>1 Officers Registered</t>
+  </si>
+  <si>
+    <t>TECHNOLOGY COMMERCIALISATION</t>
+  </si>
+  <si>
+    <t>CHEOPS TECHNOLOGY FRANCE</t>
+  </si>
+  <si>
+    <t>415050681</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>1998-01-05</t>
+  </si>
+  <si>
+    <t>5599</t>
+  </si>
+  <si>
+    <t>37 RUE, 33610, CANEJAN, France</t>
+  </si>
+  <si>
+    <t>CANEJAN</t>
+  </si>
+  <si>
+    <t>33610</t>
+  </si>
+  <si>
+    <t>DIDIER DELHOSTE (Directeur général délégué)</t>
+  </si>
+  <si>
+    <t>63.11Z</t>
+  </si>
+  <si>
+    <t>Recherche d'entreprises (api.gouv.fr)</t>
+  </si>
+  <si>
+    <t>MANGANELLI TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>483079851</t>
+  </si>
+  <si>
+    <t>2005-06-10</t>
+  </si>
+  <si>
+    <t>5710</t>
+  </si>
+  <si>
+    <t>340 AVENUE, 59700, MARCQ-EN-BARŒUL, France</t>
+  </si>
+  <si>
+    <t>MARCQ-EN-BARŒUL</t>
+  </si>
+  <si>
+    <t>59700</t>
+  </si>
+  <si>
+    <t>VALOXY AUDIT (Commissaire aux comptes titulaire)</t>
+  </si>
+  <si>
+    <t>46.52Z</t>
+  </si>
+  <si>
+    <t>COLT TECHNOLOGY SERVICES</t>
+  </si>
+  <si>
+    <t>402628838</t>
+  </si>
+  <si>
+    <t>1995-10-18</t>
+  </si>
+  <si>
+    <t>23 RUE, 92240, MALAKOFF, France</t>
+  </si>
+  <si>
+    <t>MALAKOFF</t>
+  </si>
+  <si>
+    <t>92240</t>
+  </si>
+  <si>
+    <t>MAHER EL FEKIH (Président de SAS)</t>
+  </si>
+  <si>
+    <t>61.10Z</t>
+  </si>
+  <si>
+    <t>VOI TECHNOLOGY SASU</t>
+  </si>
+  <si>
+    <t>844614248</t>
+  </si>
+  <si>
+    <t>2018-12-10</t>
+  </si>
+  <si>
+    <t>40 RUE, 75001, PARIS, France</t>
+  </si>
+  <si>
+    <t>PARIS</t>
+  </si>
+  <si>
+    <t>75001</t>
+  </si>
+  <si>
+    <t>AB CONSULTING (Commissaire aux comptes suppléant)</t>
+  </si>
+  <si>
+    <t>77.21Z</t>
+  </si>
+  <si>
+    <t>SECURITAS TECHNOLOGY SERVICES SAS</t>
+  </si>
+  <si>
+    <t>702034448</t>
+  </si>
+  <si>
+    <t>1970-01-01</t>
+  </si>
+  <si>
+    <t>253 QUAI, 92130, ISSY-LES-MOULINEAUX, France</t>
+  </si>
+  <si>
+    <t>ISSY-LES-MOULINEAUX</t>
+  </si>
+  <si>
+    <t>92130</t>
+  </si>
+  <si>
+    <t>MATTHIEU LE TAILLANDIER DE GABORY (Président de SAS)</t>
+  </si>
+  <si>
+    <t>80.20Z</t>
+  </si>
+  <si>
+    <t>C-TECHNOLOGY (PEAKSYS)</t>
+  </si>
+  <si>
+    <t>879879260</t>
+  </si>
+  <si>
+    <t>2019-12-09</t>
+  </si>
+  <si>
+    <t>120 QUAI, 33300, BORDEAUX, France</t>
+  </si>
+  <si>
+    <t>BORDEAUX</t>
+  </si>
+  <si>
+    <t>33300</t>
+  </si>
+  <si>
+    <t>THOMAS PASCAL XISTE METIVIER (Président de SAS)</t>
+  </si>
+  <si>
+    <t>62.01Z</t>
+  </si>
+  <si>
+    <t>T&amp;S TECHNOLOGY &amp;STRATEGY ENGINEERING (TECHNOLOGY &amp; STRATEGY ENGINEERING)</t>
+  </si>
+  <si>
+    <t>502192149</t>
+  </si>
+  <si>
+    <t>2008-01-18</t>
+  </si>
+  <si>
+    <t>4 RUE, 67300, SCHILTIGHEIM, France</t>
+  </si>
+  <si>
+    <t>SCHILTIGHEIM</t>
+  </si>
+  <si>
+    <t>67300</t>
+  </si>
+  <si>
+    <t>SECAL (Commissaire aux comptes titulaire)</t>
+  </si>
+  <si>
+    <t>71.12B</t>
+  </si>
+  <si>
+    <t>CAPGEMINI TECHNOLOGY SERVICES</t>
+  </si>
+  <si>
+    <t>479766842</t>
+  </si>
+  <si>
+    <t>2004-11-16</t>
+  </si>
+  <si>
+    <t>145 QUAI, 92130, ISSY-LES-MOULINEAUX, France</t>
+  </si>
+  <si>
+    <t>EMMANUEL BENOIST (Commissaire aux comptes suppléant)</t>
+  </si>
+  <si>
+    <t>62.02A</t>
+  </si>
+  <si>
+    <t>FOSSE TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>930782599</t>
+  </si>
+  <si>
+    <t>Norway</t>
+  </si>
+  <si>
+    <t>2023-02-07</t>
+  </si>
+  <si>
+    <t>Enkeltpersonforetak</t>
+  </si>
+  <si>
+    <t>Hans Hauges gate 11, 5033, BERGEN, Norge</t>
+  </si>
+  <si>
+    <t>BERGEN</t>
+  </si>
+  <si>
+    <t>5033</t>
+  </si>
+  <si>
+    <t>Dataprogrammeringstjenester</t>
+  </si>
+  <si>
+    <t>Brønnøysundregistrene (data.brreg.no)</t>
+  </si>
+  <si>
+    <t>FORCE TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>980851095</t>
+  </si>
+  <si>
+    <t>1999-06-15</t>
+  </si>
+  <si>
+    <t>Utenlandsk enhet</t>
+  </si>
+  <si>
+    <t>Park Allé 345, 2605 BRØNDBY, Danmark</t>
+  </si>
+  <si>
+    <t>2605 BRØNDBY</t>
+  </si>
+  <si>
+    <t>https://force.dk</t>
+  </si>
+  <si>
+    <t>infor@forcetechnology.dk</t>
+  </si>
+  <si>
+    <t>+4543267000</t>
+  </si>
+  <si>
+    <t>FJERDINGSTAD TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>988401498</t>
+  </si>
+  <si>
+    <t>2005-06-30</t>
+  </si>
+  <si>
+    <t>Ormerudveien 10B, 1410, KOLBOTN, Norge</t>
+  </si>
+  <si>
+    <t>KOLBOTN</t>
+  </si>
+  <si>
+    <t>1410</t>
+  </si>
+  <si>
+    <t>solvef@yahoo.com</t>
+  </si>
+  <si>
+    <t>90196722</t>
+  </si>
+  <si>
+    <t>Annen teknisk konsulentvirksomhet</t>
+  </si>
+  <si>
+    <t>DJUPVIK TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>928985148</t>
+  </si>
+  <si>
+    <t>2022-03-28</t>
+  </si>
+  <si>
+    <t>Moholt alle 11, 7050, TRONDHEIM, Norge</t>
+  </si>
+  <si>
+    <t>TRONDHEIM</t>
+  </si>
+  <si>
+    <t>7050</t>
+  </si>
+  <si>
+    <t>DAGAAR TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>937481136</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>Forening/lag/innretning</t>
+  </si>
+  <si>
+    <t>Ammerudhellinga 56, 0959, OSLO, Norge</t>
+  </si>
+  <si>
+    <t>OSLO</t>
+  </si>
+  <si>
+    <t>0959</t>
+  </si>
+  <si>
+    <t>Aktiviteter i andre medlemsorganisasjoner ellers</t>
+  </si>
+  <si>
+    <t>BEYER TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>930766178</t>
+  </si>
+  <si>
+    <t>2023-02-03</t>
+  </si>
+  <si>
+    <t>Slettevegen 3, 5360, KOLLTVEIT, Norge</t>
+  </si>
+  <si>
+    <t>KOLLTVEIT</t>
+  </si>
+  <si>
+    <t>5360</t>
+  </si>
+  <si>
+    <t>BERGERSEN TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>923034854</t>
+  </si>
+  <si>
+    <t>2019-07-05</t>
+  </si>
+  <si>
+    <t>Terrasseveien 17B, 1369, STABEKK, Norge</t>
+  </si>
+  <si>
+    <t>STABEKK</t>
+  </si>
+  <si>
+    <t>1369</t>
+  </si>
+  <si>
+    <t>BARDAL TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>937448678</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>Nedre gate 8A, 0551, OSLO, Norge</t>
+  </si>
+  <si>
+    <t>0551</t>
+  </si>
+  <si>
+    <t>BADAWI TECHNOLOGY</t>
+  </si>
+  <si>
+    <t>933418057</t>
+  </si>
+  <si>
+    <t>2024-05-07</t>
+  </si>
+  <si>
+    <t>Fullriggerveien 21, 4624, KRISTIANSAND S, Norge</t>
+  </si>
+  <si>
+    <t>KRISTIANSAND S</t>
+  </si>
+  <si>
+    <t>4624</t>
+  </si>
+  <si>
+    <t>Annen virksomhet for distribuering av innhold</t>
+  </si>
+  <si>
     <t>The Steward Shipping Foundation</t>
   </si>
   <si>
     <t>19871120103</t>
   </si>
   <si>
-    <t>United States</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
     <t>1951-05-08</t>
   </si>
   <si>
@@ -88,18 +895,6 @@
     <t>80107</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Jurisdiction: CO</t>
-  </si>
-  <si>
-    <t>US Socrata Open Data (Colorado &amp; NY)</t>
-  </si>
-  <si>
-    <t>2026-10-11</t>
-  </si>
-  <si>
     <t>THE STANDARD SHALE PRODUCTS COMPANY</t>
   </si>
   <si>
@@ -130,12 +925,6 @@
     <t>1968-06-24</t>
   </si>
   <si>
-    <t>FPC</t>
-  </si>
-  <si>
-    <t>Jurisdiction: DE</t>
-  </si>
-  <si>
     <t>CONOCOPHILLIPS COMMUNICAITONS INC.</t>
   </si>
   <si>
@@ -160,18 +949,12 @@
     <t>194600008E</t>
   </si>
   <si>
-    <t>Singapore</t>
-  </si>
-  <si>
     <t>Dissolved - Members Voluntary Winding Up</t>
   </si>
   <si>
     <t>1946-08-14</t>
   </si>
   <si>
-    <t>Exempt Private Company Limited by Shares</t>
-  </si>
-  <si>
     <t>Blk 75 TANGLIN ROAD, Singapore 247917</t>
   </si>
   <si>
@@ -184,9 +967,6 @@
     <t>52222</t>
   </si>
   <si>
-    <t>ACRA (data.gov.sg)</t>
-  </si>
-  <si>
     <t>ANEKA SERVICES</t>
   </si>
   <si>
@@ -199,9 +979,6 @@
     <t>1975-07-29</t>
   </si>
   <si>
-    <t>Sole Proprietorship/ Partnership</t>
-  </si>
-  <si>
     <t>Blk 19 JALAN TENTERAM, Singapore 321019</t>
   </si>
   <si>
@@ -274,15 +1051,9 @@
     <t>831375092</t>
   </si>
   <si>
-    <t>France</t>
-  </si>
-  <si>
     <t>2017-08-01</t>
   </si>
   <si>
-    <t>5710</t>
-  </si>
-  <si>
     <t>11 RUE, 76600, LE HAVRE, France</t>
   </si>
   <si>
@@ -298,9 +1069,6 @@
     <t>64.20Z</t>
   </si>
   <si>
-    <t>Recherche d'entreprises (api.gouv.fr)</t>
-  </si>
-  <si>
     <t>SEA INVEST SHIPPING AGENCY (FRANCOIS BOYER DE LA GIRODAY - MUSO)</t>
   </si>
   <si>
@@ -397,15 +1165,9 @@
     <t>914019281</t>
   </si>
   <si>
-    <t>Norway</t>
-  </si>
-  <si>
     <t>2014-08-19</t>
   </si>
   <si>
-    <t>Forening/lag/innretning</t>
-  </si>
-  <si>
     <t>Solløkkasvingen 16, 3233, SANDEFJORD, Norge</t>
   </si>
   <si>
@@ -415,12 +1177,6 @@
     <t>3233</t>
   </si>
   <si>
-    <t>Aktiviteter i andre medlemsorganisasjoner ellers</t>
-  </si>
-  <si>
-    <t>Brønnøysundregistrene (data.brreg.no)</t>
-  </si>
-  <si>
     <t>HBV SHIPPING</t>
   </si>
   <si>
@@ -454,15 +1210,9 @@
     <t>2015-03-26</t>
   </si>
   <si>
-    <t>Enkeltpersonforetak</t>
-  </si>
-  <si>
     <t>c/o Beatrix Goovaerts Fjellstad, Vibes gate 24, 0356, OSLO, Norge</t>
   </si>
   <si>
-    <t>OSLO</t>
-  </si>
-  <si>
     <t>0356</t>
   </si>
   <si>
@@ -526,15 +1276,9 @@
     <t>2008-11-29</t>
   </si>
   <si>
-    <t>DLLC</t>
-  </si>
-  <si>
     <t>2525 S Dayton Way Apt 1210, Denver, CO, 80231, USA</t>
   </si>
   <si>
-    <t>Denver</t>
-  </si>
-  <si>
     <t>80231</t>
   </si>
   <si>
@@ -568,9 +1312,6 @@
     <t>80 RUE, 75017, PARIS, France</t>
   </si>
   <si>
-    <t>PARIS</t>
-  </si>
-  <si>
     <t>75017</t>
   </si>
   <si>
@@ -593,9 +1334,6 @@
   </si>
   <si>
     <t>5516</t>
-  </si>
-  <si>
-    <t>Dataprogrammeringstjenester</t>
   </si>
 </sst>
 </file>
@@ -1026,13 +1764,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="4" max="4" width="45" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
     <col min="7" max="7" width="45" customWidth="1"/>
@@ -1040,8 +1778,8 @@
     <col min="9" max="9" width="15" customWidth="1"/>
     <col min="10" max="10" width="45" customWidth="1"/>
     <col min="11" max="11" width="27" customWidth="1"/>
-    <col min="12" max="12" width="24" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="13" max="13" width="15" customWidth="1"/>
     <col min="14" max="14" width="45" customWidth="1"/>
     <col min="15" max="15" width="41" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
@@ -1129,30 +1867,30 @@
         <v>25</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>18</v>
@@ -1161,48 +1899,48 @@
         <v>19</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>18</v>
@@ -1211,48 +1949,48 @@
         <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>18</v>
@@ -1261,48 +1999,48 @@
         <v>19</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>18</v>
@@ -1311,990 +2049,2740 @@
         <v>19</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>49</v>
+        <v>85</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>49</v>
+        <v>85</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="D12" s="2" t="s">
-        <v>19</v>
+        <v>96</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="J12" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="O12" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="O12" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="P12" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="E13" s="3" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>19</v>
+        <v>86</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>19</v>
+        <v>96</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>19</v>
+        <v>126</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>123</v>
+        <v>85</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>103</v>
+        <v>131</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="E17" s="3" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>132</v>
+        <v>85</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>25</v>
+        <v>138</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>128</v>
+        <v>85</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>19</v>
+        <v>96</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>132</v>
+        <v>85</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>141</v>
+        <v>26</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>142</v>
+        <v>26</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>143</v>
+        <v>26</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>128</v>
+        <v>85</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>19</v>
+        <v>148</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>149</v>
+        <v>85</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>25</v>
+        <v>153</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>151</v>
+        <v>26</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>152</v>
+        <v>26</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>128</v>
+        <v>157</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>25</v>
+        <v>163</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>128</v>
+        <v>157</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="H21" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N21" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="O21" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="I21" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K21" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L21" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="M21" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="N21" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="O21" s="3" t="s">
-        <v>135</v>
-      </c>
       <c r="P21" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>18</v>
+        <v>157</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>25</v>
+        <v>181</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>26</v>
+        <v>182</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>27</v>
+        <v>165</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>49</v>
+        <v>157</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>77</v>
+        <v>185</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>62</v>
+        <v>169</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>49</v>
+        <v>187</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>73</v>
+        <v>189</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>57</v>
+        <v>165</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>87</v>
+        <v>157</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>25</v>
+        <v>197</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>128</v>
+        <v>157</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>25</v>
+        <v>205</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>135</v>
+        <v>165</v>
       </c>
       <c r="P25" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="P26" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N27" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="O27" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="P27" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="O28" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P28" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="M29" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="N29" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="O29" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="P29" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="O30" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P30" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L31" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M31" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N31" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="O31" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="P31" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="O32" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P32" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M33" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N33" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="O33" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="P33" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="O34" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P34" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M35" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N35" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="O35" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="P35" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="O36" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P36" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L37" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M37" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N37" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="O37" s="3" t="s">
         <v>28</v>
+      </c>
+      <c r="P37" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O38" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P38" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L39" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M39" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N39" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="O39" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="P39" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L41" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M41" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N41" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="O41" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="P41" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="O42" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="P42" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L43" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M43" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N43" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="O43" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="P43" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="P44" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="K45" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L45" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M45" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="O45" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="P45" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N46" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="O46" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="P46" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="J47" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K47" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L47" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M47" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N47" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="O47" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="P47" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="O48" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="P48" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="K49" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L49" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M49" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N49" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="O49" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="P49" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="O50" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="P50" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="K51" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L51" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M51" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N51" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="O51" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="P51" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M52" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N52" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="O52" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P52" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K53" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="L53" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="M53" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="N53" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="O53" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="P53" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="O54" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P54" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="J55" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K55" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L55" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M55" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N55" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="O55" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="P55" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M56" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N56" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="O56" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P56" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="J57" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K57" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L57" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M57" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N57" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="O57" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="P57" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L58" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M58" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="O58" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="P58" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="J59" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K59" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="L59" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M59" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N59" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="O59" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="P59" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M60" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N60" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="O60" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="P60" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>